<commit_message>
Remove review labels from results sheet
</commit_message>
<xml_diff>
--- a/data/CARS_IEEE_Paper_Reported_Results.xlsx
+++ b/data/CARS_IEEE_Paper_Reported_Results.xlsx
@@ -685,7 +685,7 @@
     <row r="22" ht="37" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Categories are based on source review. Items needing confirmation are marked.</t>
+          <t>Categories are based on source review.</t>
         </is>
       </c>
     </row>
@@ -997,20 +997,16 @@
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>Hallucination / Output Risk (review needed)
-Bias / Fairness (review needed)</t>
+          <t>Hallucination / Output Risk
+Bias / Fairness</t>
         </is>
       </c>
       <c r="G4" s="10" t="inlineStr">
         <is>
-          <t>Ethical / Responsible AI (review needed)</t>
-        </is>
-      </c>
-      <c r="H4" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+          <t>Ethical / Responsible AI</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="n"/>
       <c r="I4" s="10" t="inlineStr">
         <is>
           <t>Full text</t>
@@ -1045,7 +1041,7 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>Hallucination / Output Risk (review needed)</t>
+          <t>Hallucination / Output Risk</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -1053,11 +1049,7 @@
           <t>No framework recorded</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="H5" s="10" t="n"/>
       <c r="I5" s="10" t="inlineStr">
         <is>
           <t>Full text</t>
@@ -1102,15 +1094,11 @@
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>Ethical / Responsible AI (review needed)
+          <t>Ethical / Responsible AI
 Technical Controls</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="H6" s="10" t="n"/>
       <c r="I6" s="10" t="inlineStr">
         <is>
           <t>Full text</t>
@@ -1145,20 +1133,11 @@
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>Governance Drift / Visibility (review needed)
-To confirm: Data Exposure / Privacy, Compliance / Legal, Hallucination / Output Risk, IP / Confidentiality, Bias / Fairness</t>
-        </is>
-      </c>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>To confirm: NIST AI RMF, AI TRiSM, Ethical / Responsible AI, Technical Controls</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+          <t>Governance Drift / Visibility</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="n"/>
+      <c r="H7" s="10" t="n"/>
       <c r="I7" s="10" t="inlineStr">
         <is>
           <t>Abstract only</t>
@@ -1193,7 +1172,7 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>Data Exposure / Privacy (review needed)</t>
+          <t>Data Exposure / Privacy</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -1201,11 +1180,7 @@
           <t>No framework recorded</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="H8" s="10" t="n"/>
       <c r="I8" s="10" t="inlineStr">
         <is>
           <t>Full text</t>
@@ -1242,7 +1217,7 @@
         <is>
           <t>Data Exposure / Privacy
 Compliance / Legal
-Governance Drift / Visibility (review needed)
+Governance Drift / Visibility
 Bias / Fairness</t>
         </is>
       </c>
@@ -1251,11 +1226,7 @@
           <t>Ethical / Responsible AI</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="H9" s="10" t="n"/>
       <c r="I9" s="10" t="inlineStr">
         <is>
           <t>Full text</t>
@@ -1289,464 +1260,6 @@
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
-        <is>
-          <t>Data Exposure / Privacy (review needed)
-Compliance / Legal (review needed)
-Governance Drift / Visibility (review needed)
-Hallucination / Output Risk (review needed)
-IP / Confidentiality (review needed)
-Bias / Fairness (review needed)</t>
-        </is>
-      </c>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>NIST AI RMF (review needed)
-AI TRiSM (review needed)
-Ethical / Responsible AI (review needed)
-Technical Controls (review needed)</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
-      <c r="I10" s="10" t="inlineStr">
-        <is>
-          <t>Abstract and related version</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="115" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>[13]</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Managing generative AI in firms: The theory of shadow user innovation,</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>J. Waters-Lynch, D. W. E. Allen, J. Potts, and C. Berg, “Managing generative AI in firms: The theory of shadow user innovation,” SSRN, Working Paper, 2024. DOI: 10.2139/ssrn.4754950.</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=4754950</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>Research papers and reviews</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Governance Drift / Visibility (review needed)
-Bias / Fairness (review needed)
-To confirm: Data Exposure / Privacy, Compliance / Legal, Hallucination / Output Risk</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>Technical Controls (review needed)</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
-      <c r="I11" s="10" t="inlineStr">
-        <is>
-          <t>Abstract and related version</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="125" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>[16]</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Scaling enterprise AI in healthcare: The role of governance in risk mitigation frameworks,</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>A. Bodnari and J. Travis, “Scaling enterprise AI in healthcare: The role of governance in risk mitigation frameworks,” npj Digit. Med., vol. 8, 2025, Art. no. 272. DOI: 10.1038/s41746-025-01700-4.</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>https://www.nature.com/articles/s41746-025-01700-4</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>Research papers and reviews</t>
-        </is>
-      </c>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>Data Exposure / Privacy (review needed)
-Compliance / Legal (review needed)
-Hallucination / Output Risk (review needed)
-Bias / Fairness (review needed)
-To confirm: Governance Drift / Visibility</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>Ethical / Responsible AI
-Technical Controls</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
-      <c r="I12" s="10" t="inlineStr">
-        <is>
-          <t>Full text</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="115" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>[17]</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Governance of artificial intelligence: A risk and guideline-based integrative framework,</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>B. W. Wirtz, J. C. Weyerer, and I. Kehl, “Governance of artificial intelligence: A risk and guideline-based integrative framework,” Gov. Inf. Q., vol. 39, no. 4, 2022. DOI: 10.1016/j.giq.2022.101685.</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0740624X22000181</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>Research papers and reviews</t>
-        </is>
-      </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>Data Exposure / Privacy (review needed)
-Compliance / Legal (review needed)
-Bias / Fairness (review needed)
-To confirm: Governance Drift / Visibility, Hallucination / Output Risk, IP / Confidentiality</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>Ethical / Responsible AI (review needed)
-To confirm: NIST AI RMF, AI TRiSM, Technical Controls</t>
-        </is>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
-      <c r="I13" s="10" t="inlineStr">
-        <is>
-          <t>Abstract and excerpts</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="115" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>[18]</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Artificial intelligence trust, risk and security management (AI TRiSM): Frameworks, appli- cations, challenges and future research directions,</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>A. Habbal, M. K. Ali, and M. A. Abuzaraida, “Artificial intelligence trust, risk and security management (AI TRiSM): Frameworks, appli- cations, challenges and future research directions,” Expert Syst. Appl., vol. 240, p. 122442, 2024. DOI: 10.1016/j.eswa.2023.122442.</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0957417423029445</t>
-        </is>
-      </c>
-      <c r="E14" s="10" t="inlineStr">
-        <is>
-          <t>Research papers and reviews</t>
-        </is>
-      </c>
-      <c r="F14" s="10" t="inlineStr">
-        <is>
-          <t>Data Exposure / Privacy (review needed)
-Compliance / Legal (review needed)
-Bias / Fairness (review needed)
-To confirm: Governance Drift / Visibility, Hallucination / Output Risk, IP / Confidentiality</t>
-        </is>
-      </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>AI TRiSM (review needed)
-Technical Controls (review needed)
-To confirm: NIST AI RMF, Ethical / Responsible AI</t>
-        </is>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
-      <c r="I14" s="10" t="inlineStr">
-        <is>
-          <t>Abstract and excerpts</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="125" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>[19]</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Responsible artificial intelligence governance: A review and research framework,</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>E. Papagiannidis, P. Mikalef, and K. Conboy, “Responsible artificial intelligence governance: A review and research framework,” J. Strateg. Inf. Syst., vol. 34, no. 2, p. 101885, 2025. DOI: 10.1016/j.jsis.2024. 101885.</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>https://www.researchgate.net/profile/Patrick-Mikalef/publication/387997470_Responsible_artificial_intelligence_governance_A_review_and_research_framework/links/67865c7655274940f1266857/Responsible-artificial-intelligence-governance-A-review-and-research-framework.pdf</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>Research papers and reviews</t>
-        </is>
-      </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>Data Exposure / Privacy (review needed)
-Compliance / Legal (review needed)
-Hallucination / Output Risk (review needed)
-Bias / Fairness (review needed)
-To confirm: Governance Drift / Visibility</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>Ethical / Responsible AI
-Technical Controls</t>
-        </is>
-      </c>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
-      <c r="I15" s="10" t="inlineStr">
-        <is>
-          <t>Full text</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="115" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>[20]</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>A silent partner: The shadow presence of generative artificial intelligence in public administrations,</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>L. Tangi, A. P. R. Müller, and M. Combetto, “A silent partner: The shadow presence of generative artificial intelligence in public administrations,” in Electronic Participation (ePart 2025), ser. Lecture Notes in Computer Science, vol. 15978, 2026, pp. 69–86. DOI: 10. 1007/978-3-032-02515-9 5.</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>https://link.springer.com/chapter/10.1007/978-3-032-02515-9_5</t>
-        </is>
-      </c>
-      <c r="E16" s="10" t="inlineStr">
-        <is>
-          <t>Research papers and reviews</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="inlineStr">
-        <is>
-          <t>Data Exposure / Privacy
-Governance Drift / Visibility
-Hallucination / Output Risk
-Bias / Fairness</t>
-        </is>
-      </c>
-      <c r="G16" s="10" t="inlineStr">
-        <is>
-          <t>No framework recorded</t>
-        </is>
-      </c>
-      <c r="H16" s="10" t="inlineStr">
-        <is>
-          <t>Based on full text</t>
-        </is>
-      </c>
-      <c r="I16" s="10" t="inlineStr">
-        <is>
-          <t>Full text</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="115" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>[23]</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>BYOD security: A study of human dimensions,</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>K. Downer and M. Bhattacharya, “BYOD security: A study of human dimensions,” Informatics, vol. 9, no. 1, p. 16, 2022. DOI: 10.3390/ informatics9010016.</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>https://www.mdpi.com/2227-9709/9/1/16</t>
-        </is>
-      </c>
-      <c r="E17" s="10" t="inlineStr">
-        <is>
-          <t>Research papers and reviews</t>
-        </is>
-      </c>
-      <c r="F17" s="10" t="inlineStr">
-        <is>
-          <t>Not included in risk counts</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="inlineStr">
-        <is>
-          <t>Technical Controls</t>
-        </is>
-      </c>
-      <c r="H17" s="10" t="inlineStr">
-        <is>
-          <t>Based on full text</t>
-        </is>
-      </c>
-      <c r="I17" s="10" t="inlineStr">
-        <is>
-          <t>Full text</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="115" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>[25]</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Cloud security challenges and solutions: A review of current best practices,</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>A. O. Akinade, P. A. Adepoju, A. B. Ige, and A. I. Afolabi, “Cloud security challenges and solutions: A review of current best practices,” Int. J. Multidiscip. Res. Growth Eval., vol. 6, no. 1, pp. 26–35, 2025. DOI: 10.54660/.ijmrge.2025.6.1.26-35.</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="inlineStr">
-        <is>
-          <t>https://www.allmultidisciplinaryjournal.com/article/3196/download</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>Research papers and reviews</t>
-        </is>
-      </c>
-      <c r="F18" s="10" t="inlineStr">
-        <is>
-          <t>Data Exposure / Privacy (review needed)
-Compliance / Legal (review needed)
-Governance Drift / Visibility (review needed)
-IP / Confidentiality (review needed)</t>
-        </is>
-      </c>
-      <c r="G18" s="10" t="inlineStr">
-        <is>
-          <t>Technical Controls</t>
-        </is>
-      </c>
-      <c r="H18" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
-      <c r="I18" s="10" t="inlineStr">
-        <is>
-          <t>Full text</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="140" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>[28]</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>AI risk categorization decoded (AIR 2024): From government regulations to corporate policies</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>Y. Zeng et al., AI risk categorization decoded (AIR 2024): From government regulations to corporate policies, arXiv:2406.17864, 2024.</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>https://arxiv.org/abs/2406.17864</t>
-        </is>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>Research papers and reviews</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr">
         <is>
           <t>Data Exposure / Privacy
 Compliance / Legal
@@ -1756,49 +1269,420 @@
 Bias / Fairness</t>
         </is>
       </c>
-      <c r="G19" s="10" t="inlineStr">
-        <is>
-          <t>Ethical / Responsible AI (review needed)</t>
-        </is>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
-      <c r="I19" s="10" t="inlineStr">
-        <is>
-          <t>Full text</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="140" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>[29]</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>Workplace security and privacy implications in the GenAI age: A survey,</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>A. Diro et al., “Workplace security and privacy implications in the GenAI age: A survey,” J. Inf. Secur. Appl., vol. 89, p. 103960, 2025. DOI: 10.1016/j.jisa.2024.103960.</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1016/j.jisa.2024.103960</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>NIST AI RMF
+AI TRiSM
+Ethical / Responsible AI
+Technical Controls</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="n"/>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>Abstract and related version</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="115" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>[13]</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Managing generative AI in firms: The theory of shadow user innovation,</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>J. Waters-Lynch, D. W. E. Allen, J. Potts, and C. Berg, “Managing generative AI in firms: The theory of shadow user innovation,” SSRN, Working Paper, 2024. DOI: 10.2139/ssrn.4754950.</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=4754950</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>Research papers and reviews</t>
         </is>
       </c>
-      <c r="F20" s="10" t="inlineStr">
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Governance Drift / Visibility
+Bias / Fairness</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>Technical Controls</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="n"/>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>Abstract and related version</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="125" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>[16]</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Scaling enterprise AI in healthcare: The role of governance in risk mitigation frameworks,</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>A. Bodnari and J. Travis, “Scaling enterprise AI in healthcare: The role of governance in risk mitigation frameworks,” npj Digit. Med., vol. 8, 2025, Art. no. 272. DOI: 10.1038/s41746-025-01700-4.</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41746-025-01700-4</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Research papers and reviews</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Data Exposure / Privacy
+Compliance / Legal
+Hallucination / Output Risk
+Bias / Fairness</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>Ethical / Responsible AI
+Technical Controls</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="n"/>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="115" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>[17]</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Governance of artificial intelligence: A risk and guideline-based integrative framework,</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>B. W. Wirtz, J. C. Weyerer, and I. Kehl, “Governance of artificial intelligence: A risk and guideline-based integrative framework,” Gov. Inf. Q., vol. 39, no. 4, 2022. DOI: 10.1016/j.giq.2022.101685.</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>https://www.sciencedirect.com/science/article/pii/S0740624X22000181</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Research papers and reviews</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>Data Exposure / Privacy
+Compliance / Legal
+Bias / Fairness</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>Ethical / Responsible AI</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="n"/>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>Abstract and excerpts</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="115" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>[18]</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Artificial intelligence trust, risk and security management (AI TRiSM): Frameworks, appli- cations, challenges and future research directions,</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>A. Habbal, M. K. Ali, and M. A. Abuzaraida, “Artificial intelligence trust, risk and security management (AI TRiSM): Frameworks, appli- cations, challenges and future research directions,” Expert Syst. Appl., vol. 240, p. 122442, 2024. DOI: 10.1016/j.eswa.2023.122442.</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>https://www.sciencedirect.com/science/article/pii/S0957417423029445</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Research papers and reviews</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>Data Exposure / Privacy
+Compliance / Legal
+Bias / Fairness</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>AI TRiSM
+Technical Controls</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="n"/>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>Abstract and excerpts</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="125" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>[19]</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Responsible artificial intelligence governance: A review and research framework,</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>E. Papagiannidis, P. Mikalef, and K. Conboy, “Responsible artificial intelligence governance: A review and research framework,” J. Strateg. Inf. Syst., vol. 34, no. 2, p. 101885, 2025. DOI: 10.1016/j.jsis.2024. 101885.</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>https://www.researchgate.net/profile/Patrick-Mikalef/publication/387997470_Responsible_artificial_intelligence_governance_A_review_and_research_framework/links/67865c7655274940f1266857/Responsible-artificial-intelligence-governance-A-review-and-research-framework.pdf</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Research papers and reviews</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>Data Exposure / Privacy
+Compliance / Legal
+Hallucination / Output Risk
+Bias / Fairness</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>Ethical / Responsible AI
+Technical Controls</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="n"/>
+      <c r="I15" s="10" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="115" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>[20]</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>A silent partner: The shadow presence of generative artificial intelligence in public administrations,</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>L. Tangi, A. P. R. Müller, and M. Combetto, “A silent partner: The shadow presence of generative artificial intelligence in public administrations,” in Electronic Participation (ePart 2025), ser. Lecture Notes in Computer Science, vol. 15978, 2026, pp. 69–86. DOI: 10. 1007/978-3-032-02515-9 5.</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/chapter/10.1007/978-3-032-02515-9_5</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Research papers and reviews</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Data Exposure / Privacy
+Governance Drift / Visibility
+Hallucination / Output Risk
+Bias / Fairness</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>No framework recorded</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>Based on full text</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="115" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>[23]</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>BYOD security: A study of human dimensions,</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>K. Downer and M. Bhattacharya, “BYOD security: A study of human dimensions,” Informatics, vol. 9, no. 1, p. 16, 2022. DOI: 10.3390/ informatics9010016.</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>https://www.mdpi.com/2227-9709/9/1/16</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Research papers and reviews</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>Not included in risk counts</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>Technical Controls</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>Based on full text</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="115" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>[25]</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Cloud security challenges and solutions: A review of current best practices,</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>A. O. Akinade, P. A. Adepoju, A. B. Ige, and A. I. Afolabi, “Cloud security challenges and solutions: A review of current best practices,” Int. J. Multidiscip. Res. Growth Eval., vol. 6, no. 1, pp. 26–35, 2025. DOI: 10.54660/.ijmrge.2025.6.1.26-35.</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>https://www.allmultidisciplinaryjournal.com/article/3196/download</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Research papers and reviews</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>Data Exposure / Privacy
+Compliance / Legal
+Governance Drift / Visibility
+IP / Confidentiality</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>Technical Controls</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="n"/>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="140" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>[28]</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>AI risk categorization decoded (AIR 2024): From government regulations to corporate policies</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Y. Zeng et al., AI risk categorization decoded (AIR 2024): From government regulations to corporate policies, arXiv:2406.17864, 2024.</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2406.17864</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>Research papers and reviews</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
         <is>
           <t>Data Exposure / Privacy
 Compliance / Legal
@@ -1808,6 +1692,54 @@
 Bias / Fairness</t>
         </is>
       </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>Ethical / Responsible AI</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="n"/>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="140" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>[29]</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Workplace security and privacy implications in the GenAI age: A survey,</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>A. Diro et al., “Workplace security and privacy implications in the GenAI age: A survey,” J. Inf. Secur. Appl., vol. 89, p. 103960, 2025. DOI: 10.1016/j.jisa.2024.103960.</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jisa.2024.103960</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>Research papers and reviews</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>Data Exposure / Privacy
+Compliance / Legal
+Governance Drift / Visibility
+Hallucination / Output Risk
+IP / Confidentiality
+Bias / Fairness</t>
+        </is>
+      </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
           <t>Ethical / Responsible AI
@@ -1852,341 +1784,6 @@
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
-        <is>
-          <t>Data Exposure / Privacy (review needed)
-Governance Drift / Visibility (review needed)
-Hallucination / Output Risk (review needed)
-IP / Confidentiality (review needed)</t>
-        </is>
-      </c>
-      <c r="G21" s="10" t="inlineStr">
-        <is>
-          <t>Ethical / Responsible AI (review needed)</t>
-        </is>
-      </c>
-      <c r="H21" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
-      <c r="I21" s="10" t="inlineStr">
-        <is>
-          <t>Full text</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="115" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>[10]</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>Artificial intelligence risk management framework (AI RMF 1.0),</t>
-        </is>
-      </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>National Institute of Standards and Technology, “Artificial intelligence risk management framework (AI RMF 1.0),” Tech. Rep. NIST AI 100- 1, 2023. DOI: 10.6028/NIST.AI.100-1.</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.6028/NIST.AI.100-1</t>
-        </is>
-      </c>
-      <c r="E22" s="10" t="inlineStr">
-        <is>
-          <t>Frameworks and guidance</t>
-        </is>
-      </c>
-      <c r="F22" s="10" t="inlineStr">
-        <is>
-          <t>Not included in risk counts</t>
-        </is>
-      </c>
-      <c r="G22" s="10" t="inlineStr">
-        <is>
-          <t>NIST AI RMF
-Technical Controls (review needed)</t>
-        </is>
-      </c>
-      <c r="H22" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
-      <c r="I22" s="10" t="inlineStr">
-        <is>
-          <t>Full text</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="115" customHeight="1">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>[14]</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>Recommendation on the ethics of artificial intelligence,</t>
-        </is>
-      </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>UNESCO, “Recommendation on the ethics of artificial intelligence,” UNESCO, Tech. Rep., 2021. Accessed: Aug. 21, 2026. [Online]. Available: https : / / unesdoc . unesco . org / in / rest / annotationSVC / DownloadWatermarkedAttachment / attach import 75c9fb6b - 92a6 - 4982-b772-79f540c9fc39? =381137eng.pdf.</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="inlineStr">
-        <is>
-          <t>https://www.unesco.org/en/legal-affairs/recommendation-ethics-artificial-intelligence</t>
-        </is>
-      </c>
-      <c r="E23" s="10" t="inlineStr">
-        <is>
-          <t>Frameworks and guidance</t>
-        </is>
-      </c>
-      <c r="F23" s="10" t="inlineStr">
-        <is>
-          <t>Not included in risk counts</t>
-        </is>
-      </c>
-      <c r="G23" s="10" t="inlineStr">
-        <is>
-          <t>Ethical / Responsible AI</t>
-        </is>
-      </c>
-      <c r="H23" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
-      <c r="I23" s="10" t="inlineStr">
-        <is>
-          <t>Full text</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="115" customHeight="1">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>[15]</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>NIST Privacy Frame- work 1.1 (initial public draft),</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>National Institute of Standards and Technology, “NIST Privacy Frame- work 1.1 (initial public draft),” Tech. Rep. NIST CSWP 40 ipd, 2025. DOI: 10.6028/NIST.CSWP.40.ipd.</t>
-        </is>
-      </c>
-      <c r="D24" s="10" t="inlineStr">
-        <is>
-          <t>https://nvlpubs.nist.gov/nistpubs/CSWP/NIST.CSWP.40.ipd.pdf</t>
-        </is>
-      </c>
-      <c r="E24" s="10" t="inlineStr">
-        <is>
-          <t>Frameworks and guidance</t>
-        </is>
-      </c>
-      <c r="F24" s="10" t="inlineStr">
-        <is>
-          <t>Not included in risk counts</t>
-        </is>
-      </c>
-      <c r="G24" s="10" t="inlineStr">
-        <is>
-          <t>NIST AI RMF
-Technical Controls</t>
-        </is>
-      </c>
-      <c r="H24" s="10" t="inlineStr">
-        <is>
-          <t>Based on full text</t>
-        </is>
-      </c>
-      <c r="I24" s="10" t="inlineStr">
-        <is>
-          <t>Full text</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="115" customHeight="1">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>[22]</t>
-        </is>
-      </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>Risk management framework for information systems and organizations,</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>National Institute of Standards and Technology, “Risk management framework for information systems and organizations,” Tech. Rep. NIST SP 800-37 Rev. 2, 2018. DOI: 10.6028/NIST.SP.800-37r2.</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
-        <is>
-          <t>https://nvlpubs.nist.gov/nistpubs/SpecialPublications/NIST.SP.800-37r2.pdf</t>
-        </is>
-      </c>
-      <c r="E25" s="10" t="inlineStr">
-        <is>
-          <t>Frameworks and guidance</t>
-        </is>
-      </c>
-      <c r="F25" s="10" t="inlineStr">
-        <is>
-          <t>Not included in risk counts</t>
-        </is>
-      </c>
-      <c r="G25" s="10" t="inlineStr">
-        <is>
-          <t>Technical Controls</t>
-        </is>
-      </c>
-      <c r="H25" s="10" t="inlineStr">
-        <is>
-          <t>Based on full text</t>
-        </is>
-      </c>
-      <c r="I25" s="10" t="inlineStr">
-        <is>
-          <t>Full text</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="115" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>[26]</t>
-        </is>
-      </c>
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t>Artificial intelligence risk management framework: Generative AI profile,</t>
-        </is>
-      </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>National Institute of Standards and Technology, “Artificial intelligence risk management framework: Generative AI profile,” Tech. Rep. NIST AI 600-1, 2024. DOI: 10.6028/NIST.AI.600-1.</t>
-        </is>
-      </c>
-      <c r="D26" s="10" t="inlineStr">
-        <is>
-          <t>https://nvlpubs.nist.gov/nistpubs/ai/NIST.AI.600-1.pdf</t>
-        </is>
-      </c>
-      <c r="E26" s="10" t="inlineStr">
-        <is>
-          <t>Frameworks and guidance</t>
-        </is>
-      </c>
-      <c r="F26" s="10" t="inlineStr">
-        <is>
-          <t>Not included in risk counts</t>
-        </is>
-      </c>
-      <c r="G26" s="10" t="inlineStr">
-        <is>
-          <t>NIST AI RMF
-Technical Controls</t>
-        </is>
-      </c>
-      <c r="H26" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
-      <c r="I26" s="10" t="inlineStr">
-        <is>
-          <t>Full text</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="115" customHeight="1">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>[27]</t>
-        </is>
-      </c>
-      <c r="B27" s="10" t="inlineStr">
-        <is>
-          <t>OWASP Top 10 for large language model applications 2025</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>OWASP, OWASP Top 10 for large language model applications 2025, 2024. [Online]. Available: https://genai.owasp.org/llm-top-10/.</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>https://genai.owasp.org/resource/owasp-top-10-for-llm-applications-2025/</t>
-        </is>
-      </c>
-      <c r="E27" s="10" t="inlineStr">
-        <is>
-          <t>Frameworks and guidance</t>
-        </is>
-      </c>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>Not included in risk counts</t>
-        </is>
-      </c>
-      <c r="G27" s="10" t="inlineStr">
-        <is>
-          <t>Technical Controls</t>
-        </is>
-      </c>
-      <c r="H27" s="10" t="inlineStr">
-        <is>
-          <t>Based on full text</t>
-        </is>
-      </c>
-      <c r="I27" s="10" t="inlineStr">
-        <is>
-          <t>Full text</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="115" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>[7]</t>
-        </is>
-      </c>
-      <c r="B28" s="10" t="inlineStr">
-        <is>
-          <t>Bring your own AI: How to balance risks and innovation</t>
-        </is>
-      </c>
-      <c r="C28" s="10" t="inlineStr">
-        <is>
-          <t>N. van der Meulen and B. H. Wixom, Bring your own AI: How to balance risks and innovation, MIT Sloan Management Review, 2024.</t>
-        </is>
-      </c>
-      <c r="D28" s="10" t="inlineStr">
-        <is>
-          <t>https://sloanreview.mit.edu/article/bring-your-own-ai-how-to-balance-risks-and-innovation/</t>
-        </is>
-      </c>
-      <c r="E28" s="10" t="inlineStr">
-        <is>
-          <t>Professional articles and reports</t>
-        </is>
-      </c>
-      <c r="F28" s="10" t="inlineStr">
         <is>
           <t>Data Exposure / Privacy
 Governance Drift / Visibility
@@ -2194,16 +1791,331 @@
 IP / Confidentiality</t>
         </is>
       </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>Ethical / Responsible AI</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="n"/>
+      <c r="I21" s="10" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="115" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>[10]</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Artificial intelligence risk management framework (AI RMF 1.0),</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>National Institute of Standards and Technology, “Artificial intelligence risk management framework (AI RMF 1.0),” Tech. Rep. NIST AI 100- 1, 2023. DOI: 10.6028/NIST.AI.100-1.</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.6028/NIST.AI.100-1</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>Frameworks and guidance</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>Not included in risk counts</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>NIST AI RMF
+Technical Controls</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="n"/>
+      <c r="I22" s="10" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="115" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>[14]</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Recommendation on the ethics of artificial intelligence,</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>UNESCO, “Recommendation on the ethics of artificial intelligence,” UNESCO, Tech. Rep., 2021. Accessed: Aug. 21, 2026. [Online]. Available: https : / / unesdoc . unesco . org / in / rest / annotationSVC / DownloadWatermarkedAttachment / attach import 75c9fb6b - 92a6 - 4982-b772-79f540c9fc39? =381137eng.pdf.</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>https://www.unesco.org/en/legal-affairs/recommendation-ethics-artificial-intelligence</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>Frameworks and guidance</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>Not included in risk counts</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>Ethical / Responsible AI</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="n"/>
+      <c r="I23" s="10" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="115" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>[15]</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>NIST Privacy Frame- work 1.1 (initial public draft),</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>National Institute of Standards and Technology, “NIST Privacy Frame- work 1.1 (initial public draft),” Tech. Rep. NIST CSWP 40 ipd, 2025. DOI: 10.6028/NIST.CSWP.40.ipd.</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>https://nvlpubs.nist.gov/nistpubs/CSWP/NIST.CSWP.40.ipd.pdf</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>Frameworks and guidance</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>Not included in risk counts</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>NIST AI RMF
+Technical Controls</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>Based on full text</t>
+        </is>
+      </c>
+      <c r="I24" s="10" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="115" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>[22]</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Risk management framework for information systems and organizations,</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>National Institute of Standards and Technology, “Risk management framework for information systems and organizations,” Tech. Rep. NIST SP 800-37 Rev. 2, 2018. DOI: 10.6028/NIST.SP.800-37r2.</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>https://nvlpubs.nist.gov/nistpubs/SpecialPublications/NIST.SP.800-37r2.pdf</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>Frameworks and guidance</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>Not included in risk counts</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>Technical Controls</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>Based on full text</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="115" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>[26]</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Artificial intelligence risk management framework: Generative AI profile,</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>National Institute of Standards and Technology, “Artificial intelligence risk management framework: Generative AI profile,” Tech. Rep. NIST AI 600-1, 2024. DOI: 10.6028/NIST.AI.600-1.</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>https://nvlpubs.nist.gov/nistpubs/ai/NIST.AI.600-1.pdf</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>Frameworks and guidance</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>Not included in risk counts</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>NIST AI RMF
+Technical Controls</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="n"/>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="115" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>[27]</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>OWASP Top 10 for large language model applications 2025</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>OWASP, OWASP Top 10 for large language model applications 2025, 2024. [Online]. Available: https://genai.owasp.org/llm-top-10/.</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>https://genai.owasp.org/resource/owasp-top-10-for-llm-applications-2025/</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Frameworks and guidance</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>Not included in risk counts</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>Technical Controls</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>Based on full text</t>
+        </is>
+      </c>
+      <c r="I27" s="10" t="inlineStr">
+        <is>
+          <t>Full text</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="115" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>[7]</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Bring your own AI: How to balance risks and innovation</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>N. van der Meulen and B. H. Wixom, Bring your own AI: How to balance risks and innovation, MIT Sloan Management Review, 2024.</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>https://sloanreview.mit.edu/article/bring-your-own-ai-how-to-balance-risks-and-innovation/</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>Professional articles and reports</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>Data Exposure / Privacy
+Governance Drift / Visibility
+Hallucination / Output Risk
+IP / Confidentiality</t>
+        </is>
+      </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>Ethical / Responsible AI (review needed)</t>
-        </is>
-      </c>
-      <c r="H28" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+          <t>Ethical / Responsible AI</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="n"/>
       <c r="I28" s="10" t="inlineStr">
         <is>
           <t>Full text</t>
@@ -2238,21 +2150,15 @@
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>Data Exposure / Privacy (review needed)
-To confirm: Compliance / Legal, Governance Drift / Visibility, Hallucination / Output Risk, IP / Confidentiality, Bias / Fairness</t>
+          <t>Data Exposure / Privacy</t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>Technical Controls (review needed)
-To confirm: NIST AI RMF, AI TRiSM, Ethical / Responsible AI</t>
-        </is>
-      </c>
-      <c r="H29" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+          <t>Technical Controls</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="n"/>
       <c r="I29" s="10" t="inlineStr">
         <is>
           <t>Report summary; edition unconfirmed</t>
@@ -2335,21 +2241,9 @@
           <t>Background chapter</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>To confirm: Data Exposure / Privacy, Compliance / Legal, Governance Drift / Visibility, Hallucination / Output Risk, IP / Confidentiality, Bias / Fairness</t>
-        </is>
-      </c>
-      <c r="G31" s="10" t="inlineStr">
-        <is>
-          <t>To confirm: NIST AI RMF, AI TRiSM, Ethical / Responsible AI, Technical Controls</t>
-        </is>
-      </c>
-      <c r="H31" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="F31" s="10" t="n"/>
+      <c r="G31" s="10" t="n"/>
+      <c r="H31" s="10" t="n"/>
       <c r="I31" s="10" t="inlineStr">
         <is>
           <t>Abstract only</t>
@@ -2588,14 +2482,10 @@
           <t>Security challenges and ethical considerations in the adoption of generative AI technology,</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E6" s="10" t="n"/>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
@@ -2625,14 +2515,10 @@
           <t>X-Force Threat Intelligence Index 2026,</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E7" s="10" t="n"/>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>Abstract only; inclusion not confirmed</t>
+          <t>Abstract only</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -2699,11 +2585,7 @@
           <t>A review of TRiSM frameworks in artificial intelligence systems: Fundamentals, taxonomy, use cases, key challenges and future directions,</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E9" s="10" t="n"/>
       <c r="F9" s="10" t="inlineStr">
         <is>
           <t>Abstract only</t>
@@ -2736,14 +2618,10 @@
           <t>Scaling enterprise AI in healthcare: The role of governance in risk mitigation frameworks,</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E10" s="10" t="n"/>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -2773,14 +2651,10 @@
           <t>Governance of artificial intelligence: A risk and guideline-based integrative framework,</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E11" s="10" t="n"/>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>Abstract only; inclusion not confirmed</t>
+          <t>Abstract only</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
@@ -2810,14 +2684,10 @@
           <t>Artificial intelligence trust, risk and security management (AI TRiSM): Frameworks, appli- cations, challenges and future research directions,</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E12" s="10" t="n"/>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>Partial text; inclusion not confirmed</t>
+          <t>Partial text</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
@@ -2847,14 +2717,10 @@
           <t>Responsible artificial intelligence governance: A review and research framework,</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E13" s="10" t="n"/>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -2958,14 +2824,10 @@
           <t>Cloud security challenges and solutions: A review of current best practices,</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E16" s="10" t="n"/>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -3069,14 +2931,10 @@
           <t>AI invading the workplace: Negative emotions towards the organizational use of personal virtual assistants,</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E19" s="10" t="n"/>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
@@ -3180,11 +3038,7 @@
           <t>A review of TRiSM frameworks in artificial intelligence systems: Fundamentals, taxonomy, use cases, key challenges and future directions,</t>
         </is>
       </c>
-      <c r="E22" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E22" s="10" t="n"/>
       <c r="F22" s="10" t="inlineStr">
         <is>
           <t>Abstract only</t>
@@ -3217,14 +3071,10 @@
           <t>Scaling enterprise AI in healthcare: The role of governance in risk mitigation frameworks,</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E23" s="10" t="n"/>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
@@ -3254,14 +3104,10 @@
           <t>Governance of artificial intelligence: A risk and guideline-based integrative framework,</t>
         </is>
       </c>
-      <c r="E24" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E24" s="10" t="n"/>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>Abstract only; inclusion not confirmed</t>
+          <t>Abstract only</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
@@ -3291,14 +3137,10 @@
           <t>Artificial intelligence trust, risk and security management (AI TRiSM): Frameworks, appli- cations, challenges and future research directions,</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E25" s="10" t="n"/>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>Abstract only; inclusion not confirmed</t>
+          <t>Abstract only</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
@@ -3328,14 +3170,10 @@
           <t>Responsible artificial intelligence governance: A review and research framework,</t>
         </is>
       </c>
-      <c r="E26" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E26" s="10" t="n"/>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
@@ -3402,14 +3240,10 @@
           <t>Cloud security challenges and solutions: A review of current best practices,</t>
         </is>
       </c>
-      <c r="E28" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E28" s="10" t="n"/>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
@@ -3624,11 +3458,7 @@
           <t>Shadow AI: Governance, risk, and organisational resilience,</t>
         </is>
       </c>
-      <c r="E34" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E34" s="10" t="n"/>
       <c r="F34" s="10" t="inlineStr">
         <is>
           <t>Related version</t>
@@ -3698,11 +3528,7 @@
           <t>AI4People: An ethical framework for a good AI society,</t>
         </is>
       </c>
-      <c r="E36" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E36" s="10" t="n"/>
       <c r="F36" s="10" t="inlineStr">
         <is>
           <t>Category definition needs review</t>
@@ -3735,11 +3561,7 @@
           <t>A review of TRiSM frameworks in artificial intelligence systems: Fundamentals, taxonomy, use cases, key challenges and future directions,</t>
         </is>
       </c>
-      <c r="E37" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E37" s="10" t="n"/>
       <c r="F37" s="10" t="inlineStr">
         <is>
           <t>Related version</t>
@@ -3772,11 +3594,7 @@
           <t>Managing generative AI in firms: The theory of shadow user innovation,</t>
         </is>
       </c>
-      <c r="E38" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E38" s="10" t="n"/>
       <c r="F38" s="10" t="inlineStr">
         <is>
           <t>Abstract only</t>
@@ -3883,14 +3701,10 @@
           <t>Cloud security challenges and solutions: A review of current best practices,</t>
         </is>
       </c>
-      <c r="E41" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E41" s="10" t="n"/>
       <c r="F41" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G41" s="10" t="inlineStr">
@@ -3994,14 +3808,10 @@
           <t>AI invading the workplace: Negative emotions towards the organizational use of personal virtual assistants,</t>
         </is>
       </c>
-      <c r="E44" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E44" s="10" t="n"/>
       <c r="F44" s="10" t="inlineStr">
         <is>
-          <t>Category definition needs review; inclusion not confirmed</t>
+          <t>Category definition needs review</t>
         </is>
       </c>
       <c r="G44" s="10" t="inlineStr">
@@ -4068,14 +3878,10 @@
           <t>A multilevel review of artificial intelligence in organizations,</t>
         </is>
       </c>
-      <c r="E46" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E46" s="10" t="n"/>
       <c r="F46" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G46" s="10" t="inlineStr">
@@ -4105,14 +3911,10 @@
           <t>Generative AI at work,</t>
         </is>
       </c>
-      <c r="E47" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E47" s="10" t="n"/>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G47" s="10" t="inlineStr">
@@ -4216,11 +4018,7 @@
           <t>A review of TRiSM frameworks in artificial intelligence systems: Fundamentals, taxonomy, use cases, key challenges and future directions,</t>
         </is>
       </c>
-      <c r="E50" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E50" s="10" t="n"/>
       <c r="F50" s="10" t="inlineStr">
         <is>
           <t>Abstract only</t>
@@ -4253,14 +4051,10 @@
           <t>Scaling enterprise AI in healthcare: The role of governance in risk mitigation frameworks,</t>
         </is>
       </c>
-      <c r="E51" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E51" s="10" t="n"/>
       <c r="F51" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G51" s="10" t="inlineStr">
@@ -4290,14 +4084,10 @@
           <t>Responsible artificial intelligence governance: A review and research framework,</t>
         </is>
       </c>
-      <c r="E52" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E52" s="10" t="n"/>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G52" s="10" t="inlineStr">
@@ -4438,14 +4228,10 @@
           <t>AI invading the workplace: Negative emotions towards the organizational use of personal virtual assistants,</t>
         </is>
       </c>
-      <c r="E56" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E56" s="10" t="n"/>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G56" s="10" t="inlineStr">
@@ -4586,11 +4372,7 @@
           <t>A review of TRiSM frameworks in artificial intelligence systems: Fundamentals, taxonomy, use cases, key challenges and future directions,</t>
         </is>
       </c>
-      <c r="E60" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E60" s="10" t="n"/>
       <c r="F60" s="10" t="inlineStr">
         <is>
           <t>Related version</t>
@@ -4660,14 +4442,10 @@
           <t>Cloud security challenges and solutions: A review of current best practices,</t>
         </is>
       </c>
-      <c r="E62" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E62" s="10" t="n"/>
       <c r="F62" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G62" s="10" t="inlineStr">
@@ -4771,14 +4549,10 @@
           <t>AI invading the workplace: Negative emotions towards the organizational use of personal virtual assistants,</t>
         </is>
       </c>
-      <c r="E65" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E65" s="10" t="n"/>
       <c r="F65" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G65" s="10" t="inlineStr">
@@ -4808,14 +4582,10 @@
           <t>A multilevel review of artificial intelligence in organizations,</t>
         </is>
       </c>
-      <c r="E66" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E66" s="10" t="n"/>
       <c r="F66" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G66" s="10" t="inlineStr">
@@ -4919,11 +4689,7 @@
           <t>A review of TRiSM frameworks in artificial intelligence systems: Fundamentals, taxonomy, use cases, key challenges and future directions,</t>
         </is>
       </c>
-      <c r="E69" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E69" s="10" t="n"/>
       <c r="F69" s="10" t="inlineStr">
         <is>
           <t>Abstract only</t>
@@ -4956,11 +4722,7 @@
           <t>Managing generative AI in firms: The theory of shadow user innovation,</t>
         </is>
       </c>
-      <c r="E70" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E70" s="10" t="n"/>
       <c r="F70" s="10" t="inlineStr">
         <is>
           <t>Related version</t>
@@ -4993,14 +4755,10 @@
           <t>Scaling enterprise AI in healthcare: The role of governance in risk mitigation frameworks,</t>
         </is>
       </c>
-      <c r="E71" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E71" s="10" t="n"/>
       <c r="F71" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G71" s="10" t="inlineStr">
@@ -5030,14 +4788,10 @@
           <t>Governance of artificial intelligence: A risk and guideline-based integrative framework,</t>
         </is>
       </c>
-      <c r="E72" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E72" s="10" t="n"/>
       <c r="F72" s="10" t="inlineStr">
         <is>
-          <t>Partial text; inclusion not confirmed</t>
+          <t>Partial text</t>
         </is>
       </c>
       <c r="G72" s="10" t="inlineStr">
@@ -5067,14 +4821,10 @@
           <t>Artificial intelligence trust, risk and security management (AI TRiSM): Frameworks, appli- cations, challenges and future research directions,</t>
         </is>
       </c>
-      <c r="E73" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E73" s="10" t="n"/>
       <c r="F73" s="10" t="inlineStr">
         <is>
-          <t>Partial text; inclusion not confirmed</t>
+          <t>Partial text</t>
         </is>
       </c>
       <c r="G73" s="10" t="inlineStr">
@@ -5104,14 +4854,10 @@
           <t>Responsible artificial intelligence governance: A review and research framework,</t>
         </is>
       </c>
-      <c r="E74" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E74" s="10" t="n"/>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t>Full text; inclusion not confirmed</t>
+          <t>Full text</t>
         </is>
       </c>
       <c r="G74" s="10" t="inlineStr">
@@ -5289,11 +5035,7 @@
           <t>A review of TRiSM frameworks in artificial intelligence systems: Fundamentals, taxonomy, use cases, key challenges and future directions,</t>
         </is>
       </c>
-      <c r="E79" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E79" s="10" t="n"/>
       <c r="F79" s="10" t="inlineStr">
         <is>
           <t>Related version</t>
@@ -5400,11 +5142,7 @@
           <t>A review of TRiSM frameworks in artificial intelligence systems: Fundamentals, taxonomy, use cases, key challenges and future directions,</t>
         </is>
       </c>
-      <c r="E82" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E82" s="10" t="n"/>
       <c r="F82" s="10" t="inlineStr">
         <is>
           <t>Abstract only</t>
@@ -5437,11 +5175,7 @@
           <t>Artificial intelligence trust, risk and security management (AI TRiSM): Frameworks, appli- cations, challenges and future research directions,</t>
         </is>
       </c>
-      <c r="E83" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E83" s="10" t="n"/>
       <c r="F83" s="10" t="inlineStr">
         <is>
           <t>Abstract only</t>
@@ -5511,11 +5245,7 @@
           <t>A multilevel review of artificial intelligence in organizations,</t>
         </is>
       </c>
-      <c r="E85" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E85" s="10" t="n"/>
       <c r="F85" s="10" t="inlineStr">
         <is>
           <t>Category definition needs review</t>
@@ -5548,11 +5278,7 @@
           <t>The ethical and legal implications of shadow AI in sensitive industries: A focus on healthcare, finance and education,</t>
         </is>
       </c>
-      <c r="E86" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E86" s="10" t="n"/>
       <c r="F86" s="10" t="inlineStr">
         <is>
           <t>Category definition needs review</t>
@@ -5585,11 +5311,7 @@
           <t>Bring your own AI: How to balance risks and innovation</t>
         </is>
       </c>
-      <c r="E87" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E87" s="10" t="n"/>
       <c r="F87" s="10" t="inlineStr">
         <is>
           <t>Category definition needs review</t>
@@ -5659,11 +5381,7 @@
           <t>A review of TRiSM frameworks in artificial intelligence systems: Fundamentals, taxonomy, use cases, key challenges and future directions,</t>
         </is>
       </c>
-      <c r="E89" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E89" s="10" t="n"/>
       <c r="F89" s="10" t="inlineStr">
         <is>
           <t>Related version</t>
@@ -5770,11 +5488,7 @@
           <t>Governance of artificial intelligence: A risk and guideline-based integrative framework,</t>
         </is>
       </c>
-      <c r="E92" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E92" s="10" t="n"/>
       <c r="F92" s="10" t="inlineStr">
         <is>
           <t>Partial text</t>
@@ -5844,11 +5558,7 @@
           <t>AI risk categorization decoded (AIR 2024): From government regulations to corporate policies</t>
         </is>
       </c>
-      <c r="E94" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E94" s="10" t="n"/>
       <c r="F94" s="10" t="inlineStr">
         <is>
           <t>Category definition needs review</t>
@@ -5918,11 +5628,7 @@
           <t>AI invading the workplace: Negative emotions towards the organizational use of personal virtual assistants,</t>
         </is>
       </c>
-      <c r="E96" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E96" s="10" t="n"/>
       <c r="F96" s="10" t="inlineStr">
         <is>
           <t>Category definition needs review</t>
@@ -5992,11 +5698,7 @@
           <t>X-Force Threat Intelligence Index 2026,</t>
         </is>
       </c>
-      <c r="E98" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E98" s="10" t="n"/>
       <c r="F98" s="10" t="inlineStr">
         <is>
           <t>Abstract only</t>
@@ -6029,11 +5731,7 @@
           <t>Artificial intelligence risk management framework (AI RMF 1.0),</t>
         </is>
       </c>
-      <c r="E99" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E99" s="10" t="n"/>
       <c r="F99" s="10" t="inlineStr">
         <is>
           <t>Category definition needs review</t>
@@ -6066,11 +5764,7 @@
           <t>A review of TRiSM frameworks in artificial intelligence systems: Fundamentals, taxonomy, use cases, key challenges and future directions,</t>
         </is>
       </c>
-      <c r="E100" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E100" s="10" t="n"/>
       <c r="F100" s="10" t="inlineStr">
         <is>
           <t>Abstract only</t>
@@ -6103,11 +5797,7 @@
           <t>Managing generative AI in firms: The theory of shadow user innovation,</t>
         </is>
       </c>
-      <c r="E101" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E101" s="10" t="n"/>
       <c r="F101" s="10" t="inlineStr">
         <is>
           <t>Related version</t>
@@ -6214,11 +5904,7 @@
           <t>Artificial intelligence trust, risk and security management (AI TRiSM): Frameworks, appli- cations, challenges and future research directions,</t>
         </is>
       </c>
-      <c r="E104" s="10" t="inlineStr">
-        <is>
-          <t>Review needed</t>
-        </is>
-      </c>
+      <c r="E104" s="10" t="n"/>
       <c r="F104" s="10" t="inlineStr">
         <is>
           <t>Partial text</t>

</xml_diff>